<commit_message>
feat: reject shifts that start in the past
Creating, updating or importing a shift whose start (date + start time)
is already past now fails validation on "date". "Now" is Madrid time,
since shifts carry no time zone and there is no reliable country to time
zone map. The validator takes a TimeProvider so tests run on a fixed
clock, and the sample spreadsheets move to October 2027 so they keep
importing (12/10/2027 is still a national holiday in Spain and Brazil).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/turnos_ejemplo.xlsx
+++ b/samples/turnos_ejemplo.xlsx
@@ -508,7 +508,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="4">
-        <x:v>46307</x:v>
+        <x:v>46672</x:v>
       </x:c>
       <x:c r="C2" s="5">
         <x:v>0.333333333333333</x:v>
@@ -525,7 +525,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B3" s="4">
-        <x:v>46307</x:v>
+        <x:v>46672</x:v>
       </x:c>
       <x:c r="C3" s="5">
         <x:v>0.583333333333333</x:v>
@@ -542,7 +542,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="4">
-        <x:v>46307</x:v>
+        <x:v>46672</x:v>
       </x:c>
       <x:c r="C4" s="5">
         <x:v>0.916666666666667</x:v>
@@ -559,7 +559,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B5" s="4">
-        <x:v>46307</x:v>
+        <x:v>46672</x:v>
       </x:c>
       <x:c r="C5" s="5">
         <x:v>0.375</x:v>
@@ -576,7 +576,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="4">
-        <x:v>46307</x:v>
+        <x:v>46672</x:v>
       </x:c>
       <x:c r="C6" s="5">
         <x:v>0.291666666666667</x:v>
@@ -593,7 +593,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B7" s="4">
-        <x:v>46308</x:v>
+        <x:v>46673</x:v>
       </x:c>
       <x:c r="C7" s="5">
         <x:v>0.916666666666667</x:v>
@@ -610,7 +610,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="4">
-        <x:v>46308</x:v>
+        <x:v>46673</x:v>
       </x:c>
       <x:c r="C8" s="5">
         <x:v>0.333333333333333</x:v>
@@ -627,7 +627,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="4">
-        <x:v>46308</x:v>
+        <x:v>46673</x:v>
       </x:c>
       <x:c r="C9" s="5">
         <x:v>0.5</x:v>
@@ -644,7 +644,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B10" s="4">
-        <x:v>46309</x:v>
+        <x:v>46674</x:v>
       </x:c>
       <x:c r="C10" s="5">
         <x:v>0.25</x:v>

</xml_diff>